<commit_message>
Add 4P Index coding for Environmental Management Framework (School Sector Program)
Codes the Environmental Management Framework (EMF) for Nepal's School Sector Reform Plan/School Sector Program (Ministry of Education/Department of Education, ADB-financed, updating a May 2009 original), sourced from ADB's project document repository and text-extracted directly (clean text-native PDF).

4 instruments coded: the in-school plastic-product ban + hazardous-waste awareness/recycling/safe-disposal bundle, the mandatory school solid-waste segregation/disposal/composting system, the multi-level MOE-DOE-DEO-SMC institutional/monitoring mechanism, and the itemised (but 'tentative') EMF implementation budget.

Updates the combined master CSV/XLSX to include this 5th policy (33 instrument rows total across all five Nepal policies now coded) and the index README's cross-cutting notes.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/policies/4p-index/nepal-4p-index-master.xlsx
+++ b/policies/4p-index/nepal-4p-index-master.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Waste Mgmt Natl Policy 2079" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Solid Waste Mgmt Act 2068" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Sixteenth Plan 2024-29" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="EMF School Sector Program" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W30"/>
+  <dimension ref="A1:W34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3872,6 +3873,474 @@
       <c r="W30" s="2" t="inlineStr">
         <is>
           <t>Coded in force (S=1), unlike the qualitative program-level plastic/waste commitments above, because this is a specific, numerically quantified target with a fixed baseline and end-of-plan deadline that constitutes the government's own binding resource-allocation commitment -- not merely an aspirational directive to third parties. Scored as Planned government investment (0.80) per the P-scale's own example ('construction of a new waste management facility').</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="120" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Framework (EMF) for the School Sector Reform Plan (SSRP) / School Sector Program (SSP)</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adb.org/sites/default/files/project-documents/35174-082-nep-earfab.pdf</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>To integrate environmental assessment and environmental management planning into the planning, design, implementation and monitoring of school-infrastructure sub-projects under Nepal's School Sector Reform Program/School Sector Program (construction and rehabilitation of classrooms, District Education Office buildings, libraries/laboratories, toilets, water supply and seismic retrofitting), so as to identify and mitigate the adverse environmental impacts of that infrastructure work. In relation to plastics specifically, the Framework's environmental-impact mitigation table requires that solid waste (including plastic waste) generated in schools be properly segregated, minimised, reused/recycled and disposed of, and explicitly requires banning the use of plastic products in schools as a mitigation measure for hazardous-waste-related impacts.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>"Ban use of plastic products in schools." (Table: Anticipated Environmental Impacts / Mitigation Measures, row "Hazardous waste", under Section D "Anticipated Environmental Impacts"). This is a plastics-specific commitment but is not expressed as a quantified/numeric target (e.g. a percentage reduction), so Column E is coded 0.5 rather than 1.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>This is a donor-harmonised "Environmental Management Framework" (EMF) -- explicitly stated to be "equivalent to [ADB's] Environmental Assessment and Review Framework (EARF)" under ADB's 2009 Safeguard Policy Statement (footnote 2) -- prepared originally in May 2009 and updated (per this source document, ADB project document 35174-082-NEP) for the subsequent School Sector Program, with formal approval by the Ministry of Education (Table 6, item 1.1: "Approval of EMF for SSP -- MOE"). It is a programmatic safeguard framework tied to development-partner financing conditionality, not an Act of Parliament nor a Gazette-published executive regulation, so it does not qualify for the 0.75/1.0 tiers. It is coded at the higher "plan/programme incorporating quantifiable targets" tier (0.50) rather than the purely aspirational tier (0.25) because it contains multiple quantified operational elements -- an itemised implementation budget (Table 8) and monitoring indicators with defined frequencies (Tables 9-11) -- even though its specific plastics-related commitment (the in-school plastic ban) is not itself a quantified target.</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>education, waste management, health, water, construction, disaster risk management, energy</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>consumption, recycling, disposal, environmental leakage</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4, "Budgetary Requirement" / Table 8 "Cost for Implementation of EMF": a specific, itemised budget is set out for EMF implementation -- USD 5,000 for EMF translation, printing, publication and distribution; USD 25,000 for setting up a safeguard desk in DOE and DEOs; USD 100,000 for capacity building of MOE/DOE/DEOs/SMCs; environmental screening and EMP preparation costs of approximately USD 2,000 per Initial Environmental Examination (IEE) and USD 500 per Environmental Due Diligence Report (DDR), to be included in subproject costs; and environmental monitoring costs of USD 1,000 per subproject, also included in subproject costs. Coded 1 (ring-fenced) because this is a dedicated, itemised budget line created specifically for implementing this Framework's own environmental (including solid/hazardous waste) safeguard requirements.</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>0.8125</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>Consumption</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>Environmental-impact mitigation table, row "Hazardous waste" (impact: "Use [of] batteries, laboratory chemicals disposed haphazardly"): required mitigation measures are "Awareness raising on solid waste management with waste minimization, recovery and recycling. Ban use of plastic products in schools. Safe disposal of hazardous waste."</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>Responsible authorities explicit -- DOE/DEO/SMC are assigned overall EMP implementation and monitoring responsibility under Table 6 (+0.25 authority); monitoring explicit -- Table 11 (Operation Phase Monitoring), item 3, requires bi-annual monitoring of the "Solid waste management system" via "Records of waste collected and managed" by DEO/SMU, which directly covers this mitigation measure (+0.25 monitoring); the measure is stated without an exemption (+0.25 unconditional); no explicit fine or penalty is specified anywhere in the Framework for a school or implementing agency that fails to comply with this specific mitigation measure (0 enforcement).</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>Combines a Regulatory-type ban ("ban use of plastic products") with a Voluntary/persuasion element ("awareness raising ... on minimization, recovery and recycling") and a further regulatory-type safe-disposal requirement for hazardous waste generally; highest applicable score (Regulatory, 1.0) used per Coding Rule 10, with the mixed/dual nature flagged here. This is the only provision in this Framework that names "plastic" explicitly (Plastics Relevance Filter criterion (a)). No explicit enforcement mechanism (fine/penalty) is specified for non-compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="120" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Framework (EMF) for the School Sector Reform Plan (SSRP) / School Sector Program (SSP)</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adb.org/sites/default/files/project-documents/35174-082-nep-earfab.pdf</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>To integrate environmental assessment and environmental management planning into the planning, design, implementation and monitoring of school-infrastructure sub-projects under Nepal's School Sector Reform Program/School Sector Program (construction and rehabilitation of classrooms, District Education Office buildings, libraries/laboratories, toilets, water supply and seismic retrofitting), so as to identify and mitigate the adverse environmental impacts of that infrastructure work. In relation to plastics specifically, the Framework's environmental-impact mitigation table requires that solid waste (including plastic waste) generated in schools be properly segregated, minimised, reused/recycled and disposed of, and explicitly requires banning the use of plastic products in schools as a mitigation measure for hazardous-waste-related impacts.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>"Ban use of plastic products in schools." (Table: Anticipated Environmental Impacts / Mitigation Measures, row "Hazardous waste", under Section D "Anticipated Environmental Impacts"). This is a plastics-specific commitment but is not expressed as a quantified/numeric target (e.g. a percentage reduction), so Column E is coded 0.5 rather than 1.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>This is a donor-harmonised "Environmental Management Framework" (EMF) -- explicitly stated to be "equivalent to [ADB's] Environmental Assessment and Review Framework (EARF)" under ADB's 2009 Safeguard Policy Statement (footnote 2) -- prepared originally in May 2009 and updated (per this source document, ADB project document 35174-082-NEP) for the subsequent School Sector Program, with formal approval by the Ministry of Education (Table 6, item 1.1: "Approval of EMF for SSP -- MOE"). It is a programmatic safeguard framework tied to development-partner financing conditionality, not an Act of Parliament nor a Gazette-published executive regulation, so it does not qualify for the 0.75/1.0 tiers. It is coded at the higher "plan/programme incorporating quantifiable targets" tier (0.50) rather than the purely aspirational tier (0.25) because it contains multiple quantified operational elements -- an itemised implementation budget (Table 8) and monitoring indicators with defined frequencies (Tables 9-11) -- even though its specific plastics-related commitment (the in-school plastic ban) is not itself a quantified target.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>education, waste management, health, water, construction, disaster risk management, energy</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>consumption, recycling, disposal, environmental leakage</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4, "Budgetary Requirement" / Table 8 "Cost for Implementation of EMF": a specific, itemised budget is set out for EMF implementation -- USD 5,000 for EMF translation, printing, publication and distribution; USD 25,000 for setting up a safeguard desk in DOE and DEOs; USD 100,000 for capacity building of MOE/DOE/DEOs/SMCs; environmental screening and EMP preparation costs of approximately USD 2,000 per Initial Environmental Examination (IEE) and USD 500 per Environmental Due Diligence Report (DDR), to be included in subproject costs; and environmental monitoring costs of USD 1,000 per subproject, also included in subproject costs. Coded 1 (ring-fenced) because this is a dedicated, itemised budget line created specifically for implementing this Framework's own environmental (including solid/hazardous waste) safeguard requirements.</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>0.8125</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>Waste management</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Environmental-impact mitigation table, row "Solid waste management" (impact: "Spreading of waste, pungent smell, deterioration of aesthetics"): required mitigation measures are "Proper solid waste management system shall be introduced in schools with segregation of waste, and its proper disposal. Encourage composting to use in school garden."</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>Responsible authorities explicit (DOE/DEO/SMC, Table 6) (+0.25 authority); monitoring explicit -- Table 11, item 3, bi-annual monitoring of the solid waste management system via records of waste collected/managed (+0.25 monitoring); the measure is mandatory ("shall be introduced") without a stated exemption (+0.25 unconditional); no explicit fine/penalty for non-compliance (0 enforcement).</t>
+        </is>
+      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>A general mandatory school-level source-segregation and proper-disposal requirement that, in practice, applies to the plastic component of school solid waste streams (Plastics Relevance Filter criterion (c)); composting promotion is a complementary reuse-of-organics measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="120" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Framework (EMF) for the School Sector Reform Plan (SSRP) / School Sector Program (SSP)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adb.org/sites/default/files/project-documents/35174-082-nep-earfab.pdf</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>To integrate environmental assessment and environmental management planning into the planning, design, implementation and monitoring of school-infrastructure sub-projects under Nepal's School Sector Reform Program/School Sector Program (construction and rehabilitation of classrooms, District Education Office buildings, libraries/laboratories, toilets, water supply and seismic retrofitting), so as to identify and mitigate the adverse environmental impacts of that infrastructure work. In relation to plastics specifically, the Framework's environmental-impact mitigation table requires that solid waste (including plastic waste) generated in schools be properly segregated, minimised, reused/recycled and disposed of, and explicitly requires banning the use of plastic products in schools as a mitigation measure for hazardous-waste-related impacts.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>"Ban use of plastic products in schools." (Table: Anticipated Environmental Impacts / Mitigation Measures, row "Hazardous waste", under Section D "Anticipated Environmental Impacts"). This is a plastics-specific commitment but is not expressed as a quantified/numeric target (e.g. a percentage reduction), so Column E is coded 0.5 rather than 1.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>This is a donor-harmonised "Environmental Management Framework" (EMF) -- explicitly stated to be "equivalent to [ADB's] Environmental Assessment and Review Framework (EARF)" under ADB's 2009 Safeguard Policy Statement (footnote 2) -- prepared originally in May 2009 and updated (per this source document, ADB project document 35174-082-NEP) for the subsequent School Sector Program, with formal approval by the Ministry of Education (Table 6, item 1.1: "Approval of EMF for SSP -- MOE"). It is a programmatic safeguard framework tied to development-partner financing conditionality, not an Act of Parliament nor a Gazette-published executive regulation, so it does not qualify for the 0.75/1.0 tiers. It is coded at the higher "plan/programme incorporating quantifiable targets" tier (0.50) rather than the purely aspirational tier (0.25) because it contains multiple quantified operational elements -- an itemised implementation budget (Table 8) and monitoring indicators with defined frequencies (Tables 9-11) -- even though its specific plastics-related commitment (the in-school plastic ban) is not itself a quantified target.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>education, waste management, health, water, construction, disaster risk management, energy</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>consumption, recycling, disposal, environmental leakage</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4, "Budgetary Requirement" / Table 8 "Cost for Implementation of EMF": a specific, itemised budget is set out for EMF implementation -- USD 5,000 for EMF translation, printing, publication and distribution; USD 25,000 for setting up a safeguard desk in DOE and DEOs; USD 100,000 for capacity building of MOE/DOE/DEOs/SMCs; environmental screening and EMP preparation costs of approximately USD 2,000 per Initial Environmental Examination (IEE) and USD 500 per Environmental Due Diligence Report (DDR), to be included in subproject costs; and environmental monitoring costs of USD 1,000 per subproject, also included in subproject costs. Coded 1 (ring-fenced) because this is a dedicated, itemised budget line created specifically for implementing this Framework's own environmental (including solid/hazardous waste) safeguard requirements.</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>0.8125</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>Waste management</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Section F "Institutional Arrangement and Mechanism for Implementation of EMP" (Tables 6-7): establishes a multi-level implementation and compliance chain -- the Ministry of Education (MOE) as executing agency with overall coordination responsibility; the Department of Education (DOE) as implementing agency, which will recruit a full-time Environmental Officer and set up a "safeguard desk"; District Education Offices (DEOs), which will set up their own safeguard desks and conduct routine EMP monitoring; and School Management Committees (SMCs), which implement EMF requirements at the school level. DOE conducts quarterly EMP monitoring feeding into the government's quarterly portfolio review, and MOE/DOE conduct an annual central-level compliance audit.</t>
+        </is>
+      </c>
+      <c r="S33" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>Authority explicit and multi-tiered (MOE/DOE/DEO/SMC roles individually defined in Table 6) (+0.25 authority); monitoring explicit and extensive -- quarterly DOE-supervised DEO monitoring, annual MOE/DOE compliance audits, and annual reporting/feedback workshops (+0.25 monitoring); the institutional mechanism applies without a stated exemption (+0.25 unconditional); no explicit fine/penalty is specified for an implementing agency's own non-compliance with the coordination mechanism itself (0 enforcement; note a separate contract-breach remedy exists against contractors/SMC chairpersons for construction-quality issues, but that is not an environmental-compliance enforcement tool).</t>
+        </is>
+      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>0.575</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>A textbook multi-level governance coordination and institutional-setup instrument under Coding Rule 11 (national ministry -&gt; department -&gt; district office -&gt; school-level committee), scored Procedural (0.40). This is the institutional backbone through which the plastic-ban and solid-waste-management instruments above are actually implemented and monitored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="120" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Framework (EMF) for the School Sector Reform Plan (SSRP) / School Sector Program (SSP)</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adb.org/sites/default/files/project-documents/35174-082-nep-earfab.pdf</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>To integrate environmental assessment and environmental management planning into the planning, design, implementation and monitoring of school-infrastructure sub-projects under Nepal's School Sector Reform Program/School Sector Program (construction and rehabilitation of classrooms, District Education Office buildings, libraries/laboratories, toilets, water supply and seismic retrofitting), so as to identify and mitigate the adverse environmental impacts of that infrastructure work. In relation to plastics specifically, the Framework's environmental-impact mitigation table requires that solid waste (including plastic waste) generated in schools be properly segregated, minimised, reused/recycled and disposed of, and explicitly requires banning the use of plastic products in schools as a mitigation measure for hazardous-waste-related impacts.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>"Ban use of plastic products in schools." (Table: Anticipated Environmental Impacts / Mitigation Measures, row "Hazardous waste", under Section D "Anticipated Environmental Impacts"). This is a plastics-specific commitment but is not expressed as a quantified/numeric target (e.g. a percentage reduction), so Column E is coded 0.5 rather than 1.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>This is a donor-harmonised "Environmental Management Framework" (EMF) -- explicitly stated to be "equivalent to [ADB's] Environmental Assessment and Review Framework (EARF)" under ADB's 2009 Safeguard Policy Statement (footnote 2) -- prepared originally in May 2009 and updated (per this source document, ADB project document 35174-082-NEP) for the subsequent School Sector Program, with formal approval by the Ministry of Education (Table 6, item 1.1: "Approval of EMF for SSP -- MOE"). It is a programmatic safeguard framework tied to development-partner financing conditionality, not an Act of Parliament nor a Gazette-published executive regulation, so it does not qualify for the 0.75/1.0 tiers. It is coded at the higher "plan/programme incorporating quantifiable targets" tier (0.50) rather than the purely aspirational tier (0.25) because it contains multiple quantified operational elements -- an itemised implementation budget (Table 8) and monitoring indicators with defined frequencies (Tables 9-11) -- even though its specific plastics-related commitment (the in-school plastic ban) is not itself a quantified target.</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>education, waste management, health, water, construction, disaster risk management, energy</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>consumption, recycling, disposal, environmental leakage</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4, "Budgetary Requirement" / Table 8 "Cost for Implementation of EMF": a specific, itemised budget is set out for EMF implementation -- USD 5,000 for EMF translation, printing, publication and distribution; USD 25,000 for setting up a safeguard desk in DOE and DEOs; USD 100,000 for capacity building of MOE/DOE/DEOs/SMCs; environmental screening and EMP preparation costs of approximately USD 2,000 per Initial Environmental Examination (IEE) and USD 500 per Environmental Due Diligence Report (DDR), to be included in subproject costs; and environmental monitoring costs of USD 1,000 per subproject, also included in subproject costs. Coded 1 (ring-fenced) because this is a dedicated, itemised budget line created specifically for implementing this Framework's own environmental (including solid/hazardous waste) safeguard requirements.</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>0.8125</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>Waste management</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4 / Table 8 "Cost for Implementation of EMF": a specific tentative budget for EMF implementation capacity, including USD 5,000 for translation/printing/distribution, USD 25,000 for safeguard-desk setup, USD 100,000 for capacity building, and per-subproject allocations for environmental screening/assessment (~USD 2,000 per IEE, ~USD 500 per DDR) and monitoring (~USD 1,000 per subproject) -- funding that in practice supports implementation of the solid/hazardous waste (including plastic) mitigation measures identified above.</t>
+        </is>
+      </c>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>Authority explicit (DOE/MOE as budget-holder) (+0.25 authority); the budget is explicitly introduced as "tentative" and stated to "may include" the listed items ("The tentative budgetary requirement for implementation of EMF may include as presented in following Table 8"), i.e. framed as an indicative estimate rather than a firm, unconditional commitment (0 for unconditional); no monitoring mechanism is specified for tracking the budget's own execution/disbursement (0 monitoring); no enforcement mechanism attaches to under-spending or non-disbursement (0 enforcement).</t>
+        </is>
+      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="inlineStr">
+        <is>
+          <t>Scored as Planned government/donor investment (0.80) given the specific dollar-denominated capacity/implementation investment, but coded not-in-force (S=0) because of the explicit "tentative ... may include" framing, which reads as an indicative planning estimate rather than a binding allocation (Rule 12's 'may' test). This instrument-level in-force finding does not affect the separate policy-level budget coding (Column M), which asks only whether a budget/funding source is mentioned and ring-fenced -- which it is, via this same itemised table.</t>
         </is>
       </c>
     </row>
@@ -7799,4 +8268,628 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="55" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="55" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="55" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>A: policy_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>B: policy_url</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>C: policy_year</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>D: policy_objective</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>E: policy_target</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>F: policy_target_text</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>G: policy_type</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>H: policy_type_justification</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>I: policy_integration</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>J: policy_sectors_list</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>K: policy_circularity</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>L: policy_lifecycle_phases_list</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>M: policy_budget</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>N: policy_budget_text</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>O: policy_score</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>P: instrument_type</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Q: instrument_lifecycle_stage</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>R: instrument_description</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>S: instrument_in_force</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>T: instrument_implementation</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>U: instrument_implementation_text</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>V: instrument_score</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>W: comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="120" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Framework (EMF) for the School Sector Reform Plan (SSRP) / School Sector Program (SSP)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adb.org/sites/default/files/project-documents/35174-082-nep-earfab.pdf</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>To integrate environmental assessment and environmental management planning into the planning, design, implementation and monitoring of school-infrastructure sub-projects under Nepal's School Sector Reform Program/School Sector Program (construction and rehabilitation of classrooms, District Education Office buildings, libraries/laboratories, toilets, water supply and seismic retrofitting), so as to identify and mitigate the adverse environmental impacts of that infrastructure work. In relation to plastics specifically, the Framework's environmental-impact mitigation table requires that solid waste (including plastic waste) generated in schools be properly segregated, minimised, reused/recycled and disposed of, and explicitly requires banning the use of plastic products in schools as a mitigation measure for hazardous-waste-related impacts.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>"Ban use of plastic products in schools." (Table: Anticipated Environmental Impacts / Mitigation Measures, row "Hazardous waste", under Section D "Anticipated Environmental Impacts"). This is a plastics-specific commitment but is not expressed as a quantified/numeric target (e.g. a percentage reduction), so Column E is coded 0.5 rather than 1.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>This is a donor-harmonised "Environmental Management Framework" (EMF) -- explicitly stated to be "equivalent to [ADB's] Environmental Assessment and Review Framework (EARF)" under ADB's 2009 Safeguard Policy Statement (footnote 2) -- prepared originally in May 2009 and updated (per this source document, ADB project document 35174-082-NEP) for the subsequent School Sector Program, with formal approval by the Ministry of Education (Table 6, item 1.1: "Approval of EMF for SSP -- MOE"). It is a programmatic safeguard framework tied to development-partner financing conditionality, not an Act of Parliament nor a Gazette-published executive regulation, so it does not qualify for the 0.75/1.0 tiers. It is coded at the higher "plan/programme incorporating quantifiable targets" tier (0.50) rather than the purely aspirational tier (0.25) because it contains multiple quantified operational elements -- an itemised implementation budget (Table 8) and monitoring indicators with defined frequencies (Tables 9-11) -- even though its specific plastics-related commitment (the in-school plastic ban) is not itself a quantified target.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>education, waste management, health, water, construction, disaster risk management, energy</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>consumption, recycling, disposal, environmental leakage</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4, "Budgetary Requirement" / Table 8 "Cost for Implementation of EMF": a specific, itemised budget is set out for EMF implementation -- USD 5,000 for EMF translation, printing, publication and distribution; USD 25,000 for setting up a safeguard desk in DOE and DEOs; USD 100,000 for capacity building of MOE/DOE/DEOs/SMCs; environmental screening and EMP preparation costs of approximately USD 2,000 per Initial Environmental Examination (IEE) and USD 500 per Environmental Due Diligence Report (DDR), to be included in subproject costs; and environmental monitoring costs of USD 1,000 per subproject, also included in subproject costs. Coded 1 (ring-fenced) because this is a dedicated, itemised budget line created specifically for implementing this Framework's own environmental (including solid/hazardous waste) safeguard requirements.</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>0.8125</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Consumption</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Environmental-impact mitigation table, row "Hazardous waste" (impact: "Use [of] batteries, laboratory chemicals disposed haphazardly"): required mitigation measures are "Awareness raising on solid waste management with waste minimization, recovery and recycling. Ban use of plastic products in schools. Safe disposal of hazardous waste."</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>Responsible authorities explicit -- DOE/DEO/SMC are assigned overall EMP implementation and monitoring responsibility under Table 6 (+0.25 authority); monitoring explicit -- Table 11 (Operation Phase Monitoring), item 3, requires bi-annual monitoring of the "Solid waste management system" via "Records of waste collected and managed" by DEO/SMU, which directly covers this mitigation measure (+0.25 monitoring); the measure is stated without an exemption (+0.25 unconditional); no explicit fine or penalty is specified anywhere in the Framework for a school or implementing agency that fails to comply with this specific mitigation measure (0 enforcement).</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>Combines a Regulatory-type ban ("ban use of plastic products") with a Voluntary/persuasion element ("awareness raising ... on minimization, recovery and recycling") and a further regulatory-type safe-disposal requirement for hazardous waste generally; highest applicable score (Regulatory, 1.0) used per Coding Rule 10, with the mixed/dual nature flagged here. This is the only provision in this Framework that names "plastic" explicitly (Plastics Relevance Filter criterion (a)). No explicit enforcement mechanism (fine/penalty) is specified for non-compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="120" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Framework (EMF) for the School Sector Reform Plan (SSRP) / School Sector Program (SSP)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adb.org/sites/default/files/project-documents/35174-082-nep-earfab.pdf</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>To integrate environmental assessment and environmental management planning into the planning, design, implementation and monitoring of school-infrastructure sub-projects under Nepal's School Sector Reform Program/School Sector Program (construction and rehabilitation of classrooms, District Education Office buildings, libraries/laboratories, toilets, water supply and seismic retrofitting), so as to identify and mitigate the adverse environmental impacts of that infrastructure work. In relation to plastics specifically, the Framework's environmental-impact mitigation table requires that solid waste (including plastic waste) generated in schools be properly segregated, minimised, reused/recycled and disposed of, and explicitly requires banning the use of plastic products in schools as a mitigation measure for hazardous-waste-related impacts.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>"Ban use of plastic products in schools." (Table: Anticipated Environmental Impacts / Mitigation Measures, row "Hazardous waste", under Section D "Anticipated Environmental Impacts"). This is a plastics-specific commitment but is not expressed as a quantified/numeric target (e.g. a percentage reduction), so Column E is coded 0.5 rather than 1.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>This is a donor-harmonised "Environmental Management Framework" (EMF) -- explicitly stated to be "equivalent to [ADB's] Environmental Assessment and Review Framework (EARF)" under ADB's 2009 Safeguard Policy Statement (footnote 2) -- prepared originally in May 2009 and updated (per this source document, ADB project document 35174-082-NEP) for the subsequent School Sector Program, with formal approval by the Ministry of Education (Table 6, item 1.1: "Approval of EMF for SSP -- MOE"). It is a programmatic safeguard framework tied to development-partner financing conditionality, not an Act of Parliament nor a Gazette-published executive regulation, so it does not qualify for the 0.75/1.0 tiers. It is coded at the higher "plan/programme incorporating quantifiable targets" tier (0.50) rather than the purely aspirational tier (0.25) because it contains multiple quantified operational elements -- an itemised implementation budget (Table 8) and monitoring indicators with defined frequencies (Tables 9-11) -- even though its specific plastics-related commitment (the in-school plastic ban) is not itself a quantified target.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>education, waste management, health, water, construction, disaster risk management, energy</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>consumption, recycling, disposal, environmental leakage</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4, "Budgetary Requirement" / Table 8 "Cost for Implementation of EMF": a specific, itemised budget is set out for EMF implementation -- USD 5,000 for EMF translation, printing, publication and distribution; USD 25,000 for setting up a safeguard desk in DOE and DEOs; USD 100,000 for capacity building of MOE/DOE/DEOs/SMCs; environmental screening and EMP preparation costs of approximately USD 2,000 per Initial Environmental Examination (IEE) and USD 500 per Environmental Due Diligence Report (DDR), to be included in subproject costs; and environmental monitoring costs of USD 1,000 per subproject, also included in subproject costs. Coded 1 (ring-fenced) because this is a dedicated, itemised budget line created specifically for implementing this Framework's own environmental (including solid/hazardous waste) safeguard requirements.</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>0.8125</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>Waste management</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Environmental-impact mitigation table, row "Solid waste management" (impact: "Spreading of waste, pungent smell, deterioration of aesthetics"): required mitigation measures are "Proper solid waste management system shall be introduced in schools with segregation of waste, and its proper disposal. Encourage composting to use in school garden."</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>Responsible authorities explicit (DOE/DEO/SMC, Table 6) (+0.25 authority); monitoring explicit -- Table 11, item 3, bi-annual monitoring of the solid waste management system via records of waste collected/managed (+0.25 monitoring); the measure is mandatory ("shall be introduced") without a stated exemption (+0.25 unconditional); no explicit fine/penalty for non-compliance (0 enforcement).</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>A general mandatory school-level source-segregation and proper-disposal requirement that, in practice, applies to the plastic component of school solid waste streams (Plastics Relevance Filter criterion (c)); composting promotion is a complementary reuse-of-organics measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Framework (EMF) for the School Sector Reform Plan (SSRP) / School Sector Program (SSP)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adb.org/sites/default/files/project-documents/35174-082-nep-earfab.pdf</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>To integrate environmental assessment and environmental management planning into the planning, design, implementation and monitoring of school-infrastructure sub-projects under Nepal's School Sector Reform Program/School Sector Program (construction and rehabilitation of classrooms, District Education Office buildings, libraries/laboratories, toilets, water supply and seismic retrofitting), so as to identify and mitigate the adverse environmental impacts of that infrastructure work. In relation to plastics specifically, the Framework's environmental-impact mitigation table requires that solid waste (including plastic waste) generated in schools be properly segregated, minimised, reused/recycled and disposed of, and explicitly requires banning the use of plastic products in schools as a mitigation measure for hazardous-waste-related impacts.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>"Ban use of plastic products in schools." (Table: Anticipated Environmental Impacts / Mitigation Measures, row "Hazardous waste", under Section D "Anticipated Environmental Impacts"). This is a plastics-specific commitment but is not expressed as a quantified/numeric target (e.g. a percentage reduction), so Column E is coded 0.5 rather than 1.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>This is a donor-harmonised "Environmental Management Framework" (EMF) -- explicitly stated to be "equivalent to [ADB's] Environmental Assessment and Review Framework (EARF)" under ADB's 2009 Safeguard Policy Statement (footnote 2) -- prepared originally in May 2009 and updated (per this source document, ADB project document 35174-082-NEP) for the subsequent School Sector Program, with formal approval by the Ministry of Education (Table 6, item 1.1: "Approval of EMF for SSP -- MOE"). It is a programmatic safeguard framework tied to development-partner financing conditionality, not an Act of Parliament nor a Gazette-published executive regulation, so it does not qualify for the 0.75/1.0 tiers. It is coded at the higher "plan/programme incorporating quantifiable targets" tier (0.50) rather than the purely aspirational tier (0.25) because it contains multiple quantified operational elements -- an itemised implementation budget (Table 8) and monitoring indicators with defined frequencies (Tables 9-11) -- even though its specific plastics-related commitment (the in-school plastic ban) is not itself a quantified target.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>education, waste management, health, water, construction, disaster risk management, energy</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>consumption, recycling, disposal, environmental leakage</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4, "Budgetary Requirement" / Table 8 "Cost for Implementation of EMF": a specific, itemised budget is set out for EMF implementation -- USD 5,000 for EMF translation, printing, publication and distribution; USD 25,000 for setting up a safeguard desk in DOE and DEOs; USD 100,000 for capacity building of MOE/DOE/DEOs/SMCs; environmental screening and EMP preparation costs of approximately USD 2,000 per Initial Environmental Examination (IEE) and USD 500 per Environmental Due Diligence Report (DDR), to be included in subproject costs; and environmental monitoring costs of USD 1,000 per subproject, also included in subproject costs. Coded 1 (ring-fenced) because this is a dedicated, itemised budget line created specifically for implementing this Framework's own environmental (including solid/hazardous waste) safeguard requirements.</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>0.8125</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Waste management</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Section F "Institutional Arrangement and Mechanism for Implementation of EMP" (Tables 6-7): establishes a multi-level implementation and compliance chain -- the Ministry of Education (MOE) as executing agency with overall coordination responsibility; the Department of Education (DOE) as implementing agency, which will recruit a full-time Environmental Officer and set up a "safeguard desk"; District Education Offices (DEOs), which will set up their own safeguard desks and conduct routine EMP monitoring; and School Management Committees (SMCs), which implement EMF requirements at the school level. DOE conducts quarterly EMP monitoring feeding into the government's quarterly portfolio review, and MOE/DOE conduct an annual central-level compliance audit.</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>Authority explicit and multi-tiered (MOE/DOE/DEO/SMC roles individually defined in Table 6) (+0.25 authority); monitoring explicit and extensive -- quarterly DOE-supervised DEO monitoring, annual MOE/DOE compliance audits, and annual reporting/feedback workshops (+0.25 monitoring); the institutional mechanism applies without a stated exemption (+0.25 unconditional); no explicit fine/penalty is specified for an implementing agency's own non-compliance with the coordination mechanism itself (0 enforcement; note a separate contract-breach remedy exists against contractors/SMC chairpersons for construction-quality issues, but that is not an environmental-compliance enforcement tool).</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>0.575</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>A textbook multi-level governance coordination and institutional-setup instrument under Coding Rule 11 (national ministry -&gt; department -&gt; district office -&gt; school-level committee), scored Procedural (0.40). This is the institutional backbone through which the plastic-ban and solid-waste-management instruments above are actually implemented and monitored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Management Framework (EMF) for the School Sector Reform Plan (SSRP) / School Sector Program (SSP)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adb.org/sites/default/files/project-documents/35174-082-nep-earfab.pdf</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>To integrate environmental assessment and environmental management planning into the planning, design, implementation and monitoring of school-infrastructure sub-projects under Nepal's School Sector Reform Program/School Sector Program (construction and rehabilitation of classrooms, District Education Office buildings, libraries/laboratories, toilets, water supply and seismic retrofitting), so as to identify and mitigate the adverse environmental impacts of that infrastructure work. In relation to plastics specifically, the Framework's environmental-impact mitigation table requires that solid waste (including plastic waste) generated in schools be properly segregated, minimised, reused/recycled and disposed of, and explicitly requires banning the use of plastic products in schools as a mitigation measure for hazardous-waste-related impacts.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>"Ban use of plastic products in schools." (Table: Anticipated Environmental Impacts / Mitigation Measures, row "Hazardous waste", under Section D "Anticipated Environmental Impacts"). This is a plastics-specific commitment but is not expressed as a quantified/numeric target (e.g. a percentage reduction), so Column E is coded 0.5 rather than 1.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>This is a donor-harmonised "Environmental Management Framework" (EMF) -- explicitly stated to be "equivalent to [ADB's] Environmental Assessment and Review Framework (EARF)" under ADB's 2009 Safeguard Policy Statement (footnote 2) -- prepared originally in May 2009 and updated (per this source document, ADB project document 35174-082-NEP) for the subsequent School Sector Program, with formal approval by the Ministry of Education (Table 6, item 1.1: "Approval of EMF for SSP -- MOE"). It is a programmatic safeguard framework tied to development-partner financing conditionality, not an Act of Parliament nor a Gazette-published executive regulation, so it does not qualify for the 0.75/1.0 tiers. It is coded at the higher "plan/programme incorporating quantifiable targets" tier (0.50) rather than the purely aspirational tier (0.25) because it contains multiple quantified operational elements -- an itemised implementation budget (Table 8) and monitoring indicators with defined frequencies (Tables 9-11) -- even though its specific plastics-related commitment (the in-school plastic ban) is not itself a quantified target.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>education, waste management, health, water, construction, disaster risk management, energy</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>consumption, recycling, disposal, environmental leakage</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4, "Budgetary Requirement" / Table 8 "Cost for Implementation of EMF": a specific, itemised budget is set out for EMF implementation -- USD 5,000 for EMF translation, printing, publication and distribution; USD 25,000 for setting up a safeguard desk in DOE and DEOs; USD 100,000 for capacity building of MOE/DOE/DEOs/SMCs; environmental screening and EMP preparation costs of approximately USD 2,000 per Initial Environmental Examination (IEE) and USD 500 per Environmental Due Diligence Report (DDR), to be included in subproject costs; and environmental monitoring costs of USD 1,000 per subproject, also included in subproject costs. Coded 1 (ring-fenced) because this is a dedicated, itemised budget line created specifically for implementing this Framework's own environmental (including solid/hazardous waste) safeguard requirements.</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>0.8125</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Waste management</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Section F.4 / Table 8 "Cost for Implementation of EMF": a specific tentative budget for EMF implementation capacity, including USD 5,000 for translation/printing/distribution, USD 25,000 for safeguard-desk setup, USD 100,000 for capacity building, and per-subproject allocations for environmental screening/assessment (~USD 2,000 per IEE, ~USD 500 per DDR) and monitoring (~USD 1,000 per subproject) -- funding that in practice supports implementation of the solid/hazardous waste (including plastic) mitigation measures identified above.</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>Authority explicit (DOE/MOE as budget-holder) (+0.25 authority); the budget is explicitly introduced as "tentative" and stated to "may include" the listed items ("The tentative budgetary requirement for implementation of EMF may include as presented in following Table 8"), i.e. framed as an indicative estimate rather than a firm, unconditional commitment (0 for unconditional); no monitoring mechanism is specified for tracking the budget's own execution/disbursement (0 monitoring); no enforcement mechanism attaches to under-spending or non-disbursement (0 enforcement).</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>Scored as Planned government/donor investment (0.80) given the specific dollar-denominated capacity/implementation investment, but coded not-in-force (S=0) because of the explicit "tentative ... may include" framing, which reads as an indicative planning estimate rather than a binding allocation (Rule 12's 'may' test). This instrument-level in-force finding does not affect the separate policy-level budget coding (Column M), which asks only whether a budget/funding source is mentioned and ring-fenced -- which it is, via this same itemised table.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>